<commit_message>
Rend la table diamètre FP2E (lettre -> diamètre) configurable dans Excel
Nouvel onglet 'Diametre_FP2E' (colonnes Lettre, Diametre) : une ligne par
couple lettre/diamètre. Une lettre acceptant plusieurs diamètres a
plusieurs lignes (ex. G -> 60 et G -> 65). Le 1er diamètre listé pour une
lettre sert de correction proposée.

- regles_config.py : défaut DEFAUT_DIAMETRE_FP2E, chargement, génération de
  l'onglet, mise à jour de la Notice.
- logique_controles.py : les contrôles FP2E (radio/télé/manuelle et suffixe)
  lisent la table depuis la configuration au lieu de la constante codée en
  dur ; l'ancien cas particulier G->60 est remplacé par 'premier diamètre
  listé', désormais piloté par la config.
- regles_anomalies.xlsx : modèle régénéré avec le nouvel onglet.
- GUIDE_INSTALLATION.md : documentation de l'onglet.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XquXS9oQJ8gyGBBpJNDeKM
</commit_message>
<xml_diff>
--- a/regles_anomalies.xlsx
+++ b/regles_anomalies.xlsx
@@ -13,6 +13,7 @@
     <sheet name="Traites_LRA_tele" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Plage_diametre" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Longueur_tete" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Diametre_FP2E" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -418,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="70" customWidth="1" min="1" max="1"/>
@@ -494,76 +495,104 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Diametre_FP2E         : diamètre(s) correspondant à chaque lettre FP2E.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Règles :</t>
-        </is>
-      </c>
+      <c r="A13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Mode = Radio, Tele ou Manuelle (selon l'onglet).</t>
+          <t>Règles :</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Une valeur vide dans 'Type Compteur' (onglet Longueur_tete) = s'applique</t>
+          <t xml:space="preserve">  - Mode = Radio, Tele ou Manuelle (selon l'onglet).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">    à toutes les valeurs de la marque. Une ligne avec un Type précis est</t>
+          <t xml:space="preserve">  - Une valeur vide dans 'Type Compteur' (onglet Longueur_tete) = s'applique</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">    prioritaire sur la ligne générale.</t>
+          <t xml:space="preserve">    à toutes les valeurs de la marque. Une ligne avec un Type précis est</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Ne renommez PAS les onglets ni les colonnes (en-têtes).</t>
+          <t xml:space="preserve">    prioritaire sur la ligne générale.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - En cas d'erreur de saisie, l'application ignore la partie concernée et</t>
+          <t xml:space="preserve">  - Onglet Diametre_FP2E : une ligne par (Lettre, Diametre). Une lettre qui</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">    utilise les valeurs par défaut (elle ne plante pas).</t>
+          <t xml:space="preserve">    accepte plusieurs diamètres a plusieurs lignes (ex. G -&gt; 60 et G -&gt; 65).</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr"/>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Le 1er diamètre listé pour une lettre sert de correction proposée.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Astuce : pour repartir de zéro, supprimez ce fichier et relancez l'application :</t>
+          <t xml:space="preserve">  - Ne renommez PAS les onglets ni les colonnes (en-têtes).</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - En cas d'erreur de saisie, l'application ignore la partie concernée et</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    utilise les valeurs par défaut (elle ne plante pas).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Astuce : pour repartir de zéro, supprimez ce fichier et relancez l'application :</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
         <is>
           <t>il sera recréé avec les valeurs par défaut.</t>
         </is>
@@ -1347,4 +1376,214 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Lettre</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Diametre</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>400</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Ajoute la règle de longueur de tête SAPPEL INT3 (télé) = 15 caractères
En télérelève, un compteur de marque SAPPEL (C) ou SAPPEL (H) avec le
Type Compteur INT3 doit avoir un numéro de tête de 15 caractères. Ajouté
à l'onglet configurable Longueur_tete (defaut + modèle regles_anomalies.xlsx).
Les autres codes module (KM21, MAG1...) restent inchangés.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XquXS9oQJ8gyGBBpJNDeKM
</commit_message>
<xml_diff>
--- a/regles_anomalies.xlsx
+++ b/regles_anomalies.xlsx
@@ -1214,7 +1214,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1365,11 +1365,51 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>SAPPEL (C)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>INT3</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Tele</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>SAPPEL (H)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>INT3</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Tele</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
           <t>ITRON</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="n">
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="n">
         <v>8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Renommage en « Korrect'eau » + correction diamètre G = 65 en priorité
- Renommage du logiciel en « Korrect'eau » (titre de fenêtre, en-tête,
  docstrings, README, guide). L'exécutable/spec est nommé « Korrecteau »
  (sans apostrophe, pour un nom de fichier robuste).
- Diamètre FP2E lettre G : 65 devient la correction proposée en priorité
  (65 et 60 restent tous deux valides). Onglet Diametre_FP2E réordonné,
  valeur par défaut et documentation mises à jour.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MNBAg3ANVSBwWZxw9AfDaE
</commit_message>
<xml_diff>
--- a/regles_anomalies.xlsx
+++ b/regles_anomalies.xlsx
@@ -651,8 +651,6 @@
           <t>SAPPEL (C)</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -660,8 +658,6 @@
           <t>SAPPEL (H)</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -669,8 +665,6 @@
           <t>ITRON</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4311,7 +4305,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>60</v>
+        <v>65</v>
       </c>
     </row>
     <row r="10">
@@ -4321,7 +4315,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
     </row>
     <row r="11">
@@ -4451,13 +4445,11 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
           <t>KAMSTRUP</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
         <v>8</v>
       </c>
@@ -4504,8 +4496,6 @@
           <t>KAMSTRUP</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>WMS</t>

</xml_diff>

<commit_message>
Marques autorisées en Manuelle + contrôle associé
- regles_config.py : ajout du mode "Manuelle" dans Marques_autorisees
  (U KAMSTRUP, INTEGRA, SAPPEL (C), SENSUS, SAPPEL (H), ITRON, KAIFA, KAMSTRUP,
  KROHNE, ZENNER) et chargement du mode Manuelle depuis l'Excel.
- logique_controles.py : nouveau contrôle « Marque non autorisée en manuelle »
  dans check_data_manuelle (actif seulement si la liste est renseignée).
- regles_anomalies.xlsx : ajout des 10 marques Manuelle (onglets existants
  préservés).
- main.py : surlignage de la nouvelle anomalie.

Note : la colonne Mode de l'onglet accepte indifféremment les formes courtes
(Radio/Tele/Manuelle) ou complètes (Radiorelève/Télérelève/Manuelle) — la
comparaison est normalisée.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MNBAg3ANVSBwWZxw9AfDaE
</commit_message>
<xml_diff>
--- a/regles_anomalies.xlsx
+++ b/regles_anomalies.xlsx
@@ -677,7 +677,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -825,6 +825,126 @@
       <c r="B12" t="inlineStr">
         <is>
           <t>U Kamstrup</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Manuelle</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>U KAMSTRUP</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Manuelle</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>INTEGRA</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Manuelle</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>SAPPEL (C)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Manuelle</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>SENSUS</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Manuelle</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>SAPPEL (H)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Manuelle</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ITRON</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Manuelle</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>KAIFA</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Manuelle</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>KAMSTRUP</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Manuelle</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>KROHNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Manuelle</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ZENNER</t>
         </is>
       </c>
     </row>

</xml_diff>